<commit_message>
Switched sessions 3 & 4
</commit_message>
<xml_diff>
--- a/_data/sessions.xlsx
+++ b/_data/sessions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nathan/Github/jirelations/25judentum/_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF1FFF77-C3E1-2F45-A95E-CBF80D74C595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B77304CC-3F6C-4742-B144-9B514330B19C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30240" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sessions" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="72">
   <si>
     <t>blank</t>
   </si>
@@ -247,6 +247,9 @@
   </si>
   <si>
     <t>scroll.jpg</t>
+  </si>
+  <si>
+    <t>Heiligkeit, heilige Orte</t>
   </si>
 </sst>
 </file>
@@ -943,24 +946,33 @@
         <v>25</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
+      </c>
+      <c r="G5" t="s">
+        <v>56</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>40</v>
       </c>
       <c r="I5" t="str">
         <f t="shared" si="4"/>
-        <v>3. Fundamenten: Exkursion</v>
+        <v>3. Fundamenten: Tempel &amp; Synagogen</v>
       </c>
       <c r="J5" s="3">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="K5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="L5" t="str">
         <f t="shared" si="5"/>
-        <v>3-Exkursion</v>
+        <v>3-Tempel-Synagogen</v>
       </c>
       <c r="M5" s="11"/>
+      <c r="N5" s="12" t="s">
+        <v>48</v>
+      </c>
       <c r="P5" t="str">
         <f t="shared" si="2"/>
         <v>[3]</v>
@@ -990,33 +1002,28 @@
         <v>25</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G6" t="s">
-        <v>56</v>
+        <v>22</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>40</v>
+        <v>71</v>
       </c>
       <c r="I6" t="str">
         <f t="shared" si="4"/>
-        <v>4. Fundamenten: Tempel &amp; Synagogen</v>
+        <v>4. Fundamenten: Exkursion</v>
       </c>
       <c r="J6" s="3">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="K6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L6" t="str">
         <f t="shared" si="5"/>
-        <v>4-Tempel-Synagogen</v>
+        <v>4-Exkursion</v>
       </c>
       <c r="M6" s="21"/>
-      <c r="N6" s="12" t="s">
-        <v>48</v>
-      </c>
+      <c r="N6" s="12"/>
       <c r="P6" t="str">
         <f t="shared" si="2"/>
         <v>[4]</v>

</xml_diff>

<commit_message>
Slide templates & session 3
</commit_message>
<xml_diff>
--- a/_data/sessions.xlsx
+++ b/_data/sessions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nathan/Github/jirelations/25judentum/_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B77304CC-3F6C-4742-B144-9B514330B19C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82AFD192-36C8-D049-801D-9E7CE49875C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4880" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sessions" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="78">
   <si>
     <t>blank</t>
   </si>
@@ -250,6 +250,24 @@
   </si>
   <si>
     <t>Heiligkeit, heilige Orte</t>
+  </si>
+  <si>
+    <t>slide-filename</t>
+  </si>
+  <si>
+    <t>slide-frontmatter</t>
+  </si>
+  <si>
+    <t>slide-body1</t>
+  </si>
+  <si>
+    <t>slide-body2</t>
+  </si>
+  <si>
+    <t>slide-content</t>
+  </si>
+  <si>
+    <t>cohn-sherbokJudischeGlaubensuberzeugungenUnd2000</t>
   </si>
 </sst>
 </file>
@@ -715,7 +733,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q31"/>
+  <dimension ref="A1:V31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" hidden="1" customWidth="1"/>
@@ -734,9 +752,12 @@
     <col min="14" max="15" width="77.83203125" customWidth="1"/>
     <col min="16" max="16" width="12.5" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="12.5" customWidth="1"/>
+    <col min="18" max="18" width="32.5" customWidth="1"/>
+    <col min="19" max="19" width="39.6640625" customWidth="1"/>
+    <col min="20" max="20" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -788,8 +809,23 @@
       <c r="Q1" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="3">
         <v>1</v>
       </c>
@@ -846,8 +882,105 @@
 level: overview
 ---</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R2" t="str">
+        <f>_xlfn.REGEXREPLACE(D2,"\.md","-slides.md")</f>
+        <v>2025-04-24-1-slides.md</v>
+      </c>
+      <c r="S2" t="str">
+        <f>"---
+layout: reveal
+title: '"&amp;G2&amp;"'
+author: 'Nathan Gibson'
+session: "&amp;B2&amp;"
+tags: ["&amp;B2&amp;",slides]
+category: slides
+image: "&amp;K2&amp;"
+parallaxBackgroundImage: 'assets/img/"&amp;K2&amp;"'
+---
+"</f>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Was bedeutet es, jüdisch zu sein?'
+author: 'Nathan Gibson'
+session: 1
+tags: [1,slides]
+category: slides
+image: tallit-boy.jpg
+parallaxBackgroundImage: 'assets/img/tallit-boy.jpg'
+---
+</v>
+      </c>
+      <c r="T2" t="str">
+        <f>"# Einführung ins Judentum
+{: .r-fit-text}
+### "&amp;G2&amp;"
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+"&amp;N1&amp;"
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+"&amp;N2</f>
+        <v># Einführung ins Judentum
+{: .r-fit-text}
+### Was bedeutet es, jüdisch zu sein?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+objective
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+1. Über die persönlichen Ziele des Kurses nachdenken.
+2. Über einige Faktoren jüdischer Identität reflektieren.</v>
+      </c>
+      <c r="U2" t="str">
+        <f>"
+## Lektüre
+## Diskussion
+## Vorschau
+"&amp;G3</f>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
+      <c r="V2" t="str">
+        <f>_xlfn.CONCAT(S2:U2)</f>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Was bedeutet es, jüdisch zu sein?'
+author: 'Nathan Gibson'
+session: 1
+tags: [1,slides]
+category: slides
+image: tallit-boy.jpg
+parallaxBackgroundImage: 'assets/img/tallit-boy.jpg'
+---
+# Einführung ins Judentum
+{: .r-fit-text}
+### Was bedeutet es, jüdisch zu sein?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+objective
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+1. Über die persönlichen Ziele des Kurses nachdenken.
+2. Über einige Faktoren jüdischer Identität reflektieren.
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="14"/>
       <c r="C3" s="15">
         <v>45778</v>
@@ -869,8 +1002,104 @@
       </c>
       <c r="J3" s="14"/>
       <c r="N3" s="18"/>
-    </row>
-    <row r="4" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R3" t="str">
+        <f t="shared" ref="R3:R14" si="5">_xlfn.REGEXREPLACE(D3,"\.md","-slides.md")</f>
+        <v>2025-05-01-labor-day-slides.md</v>
+      </c>
+      <c r="S3" t="str">
+        <f t="shared" ref="S3:S14" si="6">"---
+layout: reveal
+title: '"&amp;G3&amp;"'
+author: 'Nathan Gibson'
+session: "&amp;B3&amp;"
+tags: ["&amp;B3&amp;",slides]
+category: slides
+image: "&amp;K3&amp;"
+parallaxBackgroundImage: 'assets/img/"&amp;K3&amp;"'
+---
+"</f>
+        <v xml:space="preserve">---
+layout: reveal
+title: ''
+author: 'Nathan Gibson'
+session: 
+tags: [,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+</v>
+      </c>
+      <c r="T3" t="str">
+        <f t="shared" ref="T3:T15" si="7">"# Einführung ins Judentum
+{: .r-fit-text}
+### "&amp;G3&amp;"
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+"&amp;N2&amp;"
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+"&amp;N3</f>
+        <v xml:space="preserve"># Einführung ins Judentum
+{: .r-fit-text}
+### 
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+1. Über die persönlichen Ziele des Kurses nachdenken.
+2. Über einige Faktoren jüdischer Identität reflektieren.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+</v>
+      </c>
+      <c r="U3" t="str">
+        <f t="shared" ref="U3:U14" si="8">"
+## Lektüre
+## Diskussion
+## Vorschau
+"&amp;G4</f>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Warum verstanden sich Israeliten als "Gottes Volk"?</v>
+      </c>
+      <c r="V3" t="str">
+        <f t="shared" ref="V3:V14" si="9">_xlfn.CONCAT(S3:U3)</f>
+        <v>---
+layout: reveal
+title: ''
+author: 'Nathan Gibson'
+session: 
+tags: [,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+# Einführung ins Judentum
+{: .r-fit-text}
+### 
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+1. Über die persönlichen Ziele des Kurses nachdenken.
+2. Über einige Faktoren jüdischer Identität reflektieren.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+## Lektüre
+## Diskussion
+## Vorschau
+Warum verstanden sich Israeliten als "Gottes Volk"?</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="3">
         <v>2</v>
       </c>
@@ -905,7 +1134,7 @@
         <v>66</v>
       </c>
       <c r="L4" t="str">
-        <f t="shared" ref="L4:L15" si="5">SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B4 &amp; ". " &amp; F4,".",""),"&amp;","")," ","-"),"--","-")</f>
+        <f t="shared" ref="L4:L15" si="10">SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B4 &amp; ". " &amp; F4,".",""),"&amp;","")," ","-"),"--","-")</f>
         <v>2-Thora-Bund</v>
       </c>
       <c r="M4" s="21" t="s">
@@ -930,8 +1159,76 @@
 level: overview
 ---</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R4" t="str">
+        <f t="shared" si="5"/>
+        <v>2025-05-08-2-slides.md</v>
+      </c>
+      <c r="S4" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Warum verstanden sich Israeliten als "Gottes Volk"?'
+author: 'Nathan Gibson'
+session: 2
+tags: [2,slides]
+category: slides
+image: dura-europos-moses-sea.jpg
+parallaxBackgroundImage: 'assets/img/dura-europos-moses-sea.jpg'
+---
+</v>
+      </c>
+      <c r="T4" t="str">
+        <f t="shared" si="7"/>
+        <v># Einführung ins Judentum
+{: .r-fit-text}
+### Warum verstanden sich Israeliten als "Gottes Volk"?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Kernbegriffe jüdischen Selbstverständnisses auf Basis der Bibel skizzieren.</v>
+      </c>
+      <c r="U4" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Welche Bedeutung haben die Form und der Ort der Anbetung?</v>
+      </c>
+      <c r="V4" t="str">
+        <f t="shared" si="9"/>
+        <v>---
+layout: reveal
+title: 'Warum verstanden sich Israeliten als "Gottes Volk"?'
+author: 'Nathan Gibson'
+session: 2
+tags: [2,slides]
+category: slides
+image: dura-europos-moses-sea.jpg
+parallaxBackgroundImage: 'assets/img/dura-europos-moses-sea.jpg'
+---
+# Einführung ins Judentum
+{: .r-fit-text}
+### Warum verstanden sich Israeliten als "Gottes Volk"?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Kernbegriffe jüdischen Selbstverständnisses auf Basis der Bibel skizzieren.
+## Lektüre
+## Diskussion
+## Vorschau
+Welche Bedeutung haben die Form und der Ort der Anbetung?</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="3">
         <v>3</v>
       </c>
@@ -966,10 +1263,12 @@
         <v>65</v>
       </c>
       <c r="L5" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v>3-Tempel-Synagogen</v>
       </c>
-      <c r="M5" s="11"/>
+      <c r="M5" s="11" t="s">
+        <v>77</v>
+      </c>
       <c r="N5" s="12" t="s">
         <v>48</v>
       </c>
@@ -986,8 +1285,78 @@
 level: overview
 ---</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R5" t="str">
+        <f t="shared" si="5"/>
+        <v>2025-05-15-3-slides.md</v>
+      </c>
+      <c r="S5" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Welche Bedeutung haben die Form und der Ort der Anbetung?'
+author: 'Nathan Gibson'
+session: 3
+tags: [3,slides]
+category: slides
+image: dura-europos-synagogue-well.jpg
+parallaxBackgroundImage: 'assets/img/dura-europos-synagogue-well.jpg'
+---
+</v>
+      </c>
+      <c r="T5" t="str">
+        <f t="shared" si="7"/>
+        <v># Einführung ins Judentum
+{: .r-fit-text}
+### Welche Bedeutung haben die Form und der Ort der Anbetung?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Kernbegriffe jüdischen Selbstverständnisses auf Basis der Bibel skizzieren.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Antike israelitische und jüdische Heiligkeitskonzepte in Bezug auf Gebetsorte und Rituale erläutern.</v>
+      </c>
+      <c r="U5" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
+      <c r="V5" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Welche Bedeutung haben die Form und der Ort der Anbetung?'
+author: 'Nathan Gibson'
+session: 3
+tags: [3,slides]
+category: slides
+image: dura-europos-synagogue-well.jpg
+parallaxBackgroundImage: 'assets/img/dura-europos-synagogue-well.jpg'
+---
+# Einführung ins Judentum
+{: .r-fit-text}
+### Welche Bedeutung haben die Form und der Ort der Anbetung?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Kernbegriffe jüdischen Selbstverständnisses auf Basis der Bibel skizzieren.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Antike israelitische und jüdische Heiligkeitskonzepte in Bezug auf Gebetsorte und Rituale erläutern.
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="3">
         <v>4</v>
       </c>
@@ -1019,7 +1388,7 @@
         <v>67</v>
       </c>
       <c r="L6" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v>4-Exkursion</v>
       </c>
       <c r="M6" s="21"/>
@@ -1037,8 +1406,77 @@
 level: overview
 ---</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R6" t="str">
+        <f t="shared" si="5"/>
+        <v>2025-05-22-4-slides.md</v>
+      </c>
+      <c r="S6" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: ''
+author: 'Nathan Gibson'
+session: 4
+tags: [4,slides]
+category: slides
+image: menorah-budapest.jpg
+parallaxBackgroundImage: 'assets/img/menorah-budapest.jpg'
+---
+</v>
+      </c>
+      <c r="T6" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve"># Einführung ins Judentum
+{: .r-fit-text}
+### 
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Antike israelitische und jüdische Heiligkeitskonzepte in Bezug auf Gebetsorte und Rituale erläutern.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+</v>
+      </c>
+      <c r="U6" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
+      <c r="V6" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: ''
+author: 'Nathan Gibson'
+session: 4
+tags: [4,slides]
+category: slides
+image: menorah-budapest.jpg
+parallaxBackgroundImage: 'assets/img/menorah-budapest.jpg'
+---
+# Einführung ins Judentum
+{: .r-fit-text}
+### 
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Antike israelitische und jüdische Heiligkeitskonzepte in Bezug auf Gebetsorte und Rituale erläutern.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="14"/>
       <c r="C7" s="15">
         <v>45806</v>
@@ -1058,8 +1496,75 @@
         <v>. Christi Himmelfahrt (vorlesungsfrei): Christi Himmelfahrt (vorlesungsfrei)</v>
       </c>
       <c r="J7" s="14"/>
-    </row>
-    <row r="8" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R7" t="str">
+        <f t="shared" si="5"/>
+        <v>2025-05-29-ascension-slides.md</v>
+      </c>
+      <c r="S7" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: ''
+author: 'Nathan Gibson'
+session: 
+tags: [,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+</v>
+      </c>
+      <c r="T7" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve"># Einführung ins Judentum
+{: .r-fit-text}
+### 
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+</v>
+      </c>
+      <c r="U7" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Wie werden die heiligen Schriften ausgelegt (und von wem)?</v>
+      </c>
+      <c r="V7" t="str">
+        <f t="shared" si="9"/>
+        <v>---
+layout: reveal
+title: ''
+author: 'Nathan Gibson'
+session: 
+tags: [,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+# Einführung ins Judentum
+{: .r-fit-text}
+### 
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+## Lektüre
+## Diskussion
+## Vorschau
+Wie werden die heiligen Schriften ausgelegt (und von wem)?</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="3">
         <v>5</v>
       </c>
@@ -1114,8 +1619,76 @@
 level: overview
 ---</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R8" t="str">
+        <f t="shared" si="5"/>
+        <v>2025-06-05-5-slides.md</v>
+      </c>
+      <c r="S8" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie werden die heiligen Schriften ausgelegt (und von wem)?'
+author: 'Nathan Gibson'
+session: 5
+tags: [5,slides]
+category: slides
+image: mishnah-frankfurt.jpg
+parallaxBackgroundImage: 'assets/img/mishnah-frankfurt.jpg'
+---
+</v>
+      </c>
+      <c r="T8" t="str">
+        <f t="shared" si="7"/>
+        <v># Einführung ins Judentum
+{: .r-fit-text}
+### Wie werden die heiligen Schriften ausgelegt (und von wem)?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Einige jüdische sakrale Texte aufzählen und ihr Zusammenspiel mit mündlichen Praktiken erläutern.</v>
+      </c>
+      <c r="U8" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Wie gestaltete sich jüdisches Leben in der Diaspora?</v>
+      </c>
+      <c r="V8" t="str">
+        <f t="shared" si="9"/>
+        <v>---
+layout: reveal
+title: 'Wie werden die heiligen Schriften ausgelegt (und von wem)?'
+author: 'Nathan Gibson'
+session: 5
+tags: [5,slides]
+category: slides
+image: mishnah-frankfurt.jpg
+parallaxBackgroundImage: 'assets/img/mishnah-frankfurt.jpg'
+---
+# Einführung ins Judentum
+{: .r-fit-text}
+### Wie werden die heiligen Schriften ausgelegt (und von wem)?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Einige jüdische sakrale Texte aufzählen und ihr Zusammenspiel mit mündlichen Praktiken erläutern.
+## Lektüre
+## Diskussion
+## Vorschau
+Wie gestaltete sich jüdisches Leben in der Diaspora?</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="3">
         <v>6</v>
       </c>
@@ -1170,8 +1743,78 @@
 level: overview
 ---</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R9" t="str">
+        <f t="shared" si="5"/>
+        <v>2025-06-12-6-slides.md</v>
+      </c>
+      <c r="S9" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie gestaltete sich jüdisches Leben in der Diaspora?'
+author: 'Nathan Gibson'
+session: 6
+tags: [6,slides]
+category: slides
+image: beit-alpha-zodiac.jpg
+parallaxBackgroundImage: 'assets/img/beit-alpha-zodiac.jpg'
+---
+</v>
+      </c>
+      <c r="T9" t="str">
+        <f t="shared" si="7"/>
+        <v># Einführung ins Judentum
+{: .r-fit-text}
+### Wie gestaltete sich jüdisches Leben in der Diaspora?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Einige jüdische sakrale Texte aufzählen und ihr Zusammenspiel mit mündlichen Praktiken erläutern.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Beispiele für die Folgen des sprachlichen und kulturellen Kontakts mit dem Aramäischen und Griechischen nennen.</v>
+      </c>
+      <c r="U9" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
+      <c r="V9" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie gestaltete sich jüdisches Leben in der Diaspora?'
+author: 'Nathan Gibson'
+session: 6
+tags: [6,slides]
+category: slides
+image: beit-alpha-zodiac.jpg
+parallaxBackgroundImage: 'assets/img/beit-alpha-zodiac.jpg'
+---
+# Einführung ins Judentum
+{: .r-fit-text}
+### Wie gestaltete sich jüdisches Leben in der Diaspora?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Einige jüdische sakrale Texte aufzählen und ihr Zusammenspiel mit mündlichen Praktiken erläutern.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Beispiele für die Folgen des sprachlichen und kulturellen Kontakts mit dem Aramäischen und Griechischen nennen.
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="14"/>
       <c r="C10" s="15">
         <v>45827</v>
@@ -1190,8 +1833,77 @@
         <v>. Fronleichnam (vorlesungsfrei): Fronleichnam (vorlesungsfrei)</v>
       </c>
       <c r="J10" s="14"/>
-    </row>
-    <row r="11" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R10" t="str">
+        <f t="shared" si="5"/>
+        <v>2025-06-19-corpus-christi-slides.md</v>
+      </c>
+      <c r="S10" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: ''
+author: 'Nathan Gibson'
+session: 
+tags: [,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+</v>
+      </c>
+      <c r="T10" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve"># Einführung ins Judentum
+{: .r-fit-text}
+### 
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Beispiele für die Folgen des sprachlichen und kulturellen Kontakts mit dem Aramäischen und Griechischen nennen.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+</v>
+      </c>
+      <c r="U10" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
+      <c r="V10" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: ''
+author: 'Nathan Gibson'
+session: 
+tags: [,slides]
+category: slides
+image: 
+parallaxBackgroundImage: 'assets/img/'
+---
+# Einführung ins Judentum
+{: .r-fit-text}
+### 
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Beispiele für die Folgen des sprachlichen und kulturellen Kontakts mit dem Aramäischen und Griechischen nennen.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="3">
         <v>7</v>
       </c>
@@ -1220,7 +1932,7 @@
         <v>68</v>
       </c>
       <c r="L11" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v>7-Exkursion</v>
       </c>
       <c r="M11" s="11"/>
@@ -1237,8 +1949,75 @@
 level: overview
 ---</v>
       </c>
-    </row>
-    <row r="12" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R11" t="str">
+        <f t="shared" si="5"/>
+        <v>2025-06-26-7-slides.md</v>
+      </c>
+      <c r="S11" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: ''
+author: 'Nathan Gibson'
+session: 7
+tags: [7,slides]
+category: slides
+image: torah-crown.jpg
+parallaxBackgroundImage: 'assets/img/torah-crown.jpg'
+---
+</v>
+      </c>
+      <c r="T11" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve"># Einführung ins Judentum
+{: .r-fit-text}
+### 
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+</v>
+      </c>
+      <c r="U11" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Wie haben sich Juden von anderen Monotheisten unterschieden?</v>
+      </c>
+      <c r="V11" t="str">
+        <f t="shared" si="9"/>
+        <v>---
+layout: reveal
+title: ''
+author: 'Nathan Gibson'
+session: 7
+tags: [7,slides]
+category: slides
+image: torah-crown.jpg
+parallaxBackgroundImage: 'assets/img/torah-crown.jpg'
+---
+# Einführung ins Judentum
+{: .r-fit-text}
+### 
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+## Lektüre
+## Diskussion
+## Vorschau
+Wie haben sich Juden von anderen Monotheisten unterschieden?</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="3">
         <v>8</v>
       </c>
@@ -1273,7 +2052,7 @@
         <v>61</v>
       </c>
       <c r="L12" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v>8-Juden,-Samaritaner-Gottesfürchtige</v>
       </c>
       <c r="M12" s="21"/>
@@ -1293,8 +2072,76 @@
 level: overview
 ---</v>
       </c>
-    </row>
-    <row r="13" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R12" t="str">
+        <f t="shared" si="5"/>
+        <v>2025-07-03-8-slides.md</v>
+      </c>
+      <c r="S12" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie haben sich Juden von anderen Monotheisten unterschieden?'
+author: 'Nathan Gibson'
+session: 8
+tags: [8,slides]
+category: slides
+image: 20090409-MT-gerizem-sameritan-sacrifice-highpriests-003-2.jpg
+parallaxBackgroundImage: 'assets/img/20090409-MT-gerizem-sameritan-sacrifice-highpriests-003-2.jpg'
+---
+</v>
+      </c>
+      <c r="T12" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve"># Einführung ins Judentum
+{: .r-fit-text}
+### Wie haben sich Juden von anderen Monotheisten unterschieden?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Die Entwicklung der jüdischen Selbstbestimmung skizzieren. </v>
+      </c>
+      <c r="U12" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Wie trennten sich die Wege der verschiedenen Sekten?</v>
+      </c>
+      <c r="V12" t="str">
+        <f t="shared" si="9"/>
+        <v>---
+layout: reveal
+title: 'Wie haben sich Juden von anderen Monotheisten unterschieden?'
+author: 'Nathan Gibson'
+session: 8
+tags: [8,slides]
+category: slides
+image: 20090409-MT-gerizem-sameritan-sacrifice-highpriests-003-2.jpg
+parallaxBackgroundImage: 'assets/img/20090409-MT-gerizem-sameritan-sacrifice-highpriests-003-2.jpg'
+---
+# Einführung ins Judentum
+{: .r-fit-text}
+### Wie haben sich Juden von anderen Monotheisten unterschieden?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Die Entwicklung der jüdischen Selbstbestimmung skizzieren. 
+## Lektüre
+## Diskussion
+## Vorschau
+Wie trennten sich die Wege der verschiedenen Sekten?</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="3">
         <v>9</v>
       </c>
@@ -1326,7 +2173,7 @@
         <v>63</v>
       </c>
       <c r="L13" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v>9-Rabbiner-messianische-Bewegungen</v>
       </c>
       <c r="M13" s="21"/>
@@ -1346,8 +2193,78 @@
 level: overview
 ---</v>
       </c>
-    </row>
-    <row r="14" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R13" t="str">
+        <f t="shared" si="5"/>
+        <v>2025-07-10-9-slides.md</v>
+      </c>
+      <c r="S13" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie trennten sich die Wege der verschiedenen Sekten?'
+author: 'Nathan Gibson'
+session: 9
+tags: [9,slides]
+category: slides
+image: bar-kokhba-weight.jpg
+parallaxBackgroundImage: 'assets/img/bar-kokhba-weight.jpg'
+---
+</v>
+      </c>
+      <c r="T13" t="str">
+        <f t="shared" si="7"/>
+        <v># Einführung ins Judentum
+{: .r-fit-text}
+### Wie trennten sich die Wege der verschiedenen Sekten?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Die Entwicklung der jüdischen Selbstbestimmung skizzieren. 
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Gründe nennen, warum die Rabbiner nicht als alleinige Repräsentanten des Judentums in den ersten Jahrhunderten u.Z. anzusehen sind.</v>
+      </c>
+      <c r="U13" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Wie positionierten sich Rabbiner als die Wahren gegenüber Karäern und Muslimen?</v>
+      </c>
+      <c r="V13" t="str">
+        <f t="shared" si="9"/>
+        <v>---
+layout: reveal
+title: 'Wie trennten sich die Wege der verschiedenen Sekten?'
+author: 'Nathan Gibson'
+session: 9
+tags: [9,slides]
+category: slides
+image: bar-kokhba-weight.jpg
+parallaxBackgroundImage: 'assets/img/bar-kokhba-weight.jpg'
+---
+# Einführung ins Judentum
+{: .r-fit-text}
+### Wie trennten sich die Wege der verschiedenen Sekten?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Die Entwicklung der jüdischen Selbstbestimmung skizzieren. 
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Gründe nennen, warum die Rabbiner nicht als alleinige Repräsentanten des Judentums in den ersten Jahrhunderten u.Z. anzusehen sind.
+## Lektüre
+## Diskussion
+## Vorschau
+Wie positionierten sich Rabbiner als die Wahren gegenüber Karäern und Muslimen?</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="3">
         <v>10</v>
       </c>
@@ -1379,7 +2296,7 @@
         <v>62</v>
       </c>
       <c r="L14" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v>10-Rabbiner,-Karäer-und-Muslime</v>
       </c>
       <c r="M14" s="11"/>
@@ -1399,8 +2316,78 @@
 level: overview
 ---</v>
       </c>
-    </row>
-    <row r="15" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R14" t="str">
+        <f t="shared" si="5"/>
+        <v>2025-07-17-10-slides.md</v>
+      </c>
+      <c r="S14" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Wie positionierten sich Rabbiner als die Wahren gegenüber Karäern und Muslimen?'
+author: 'Nathan Gibson'
+session: 10
+tags: [10,slides]
+category: slides
+image: torah-islamicate.jpg
+parallaxBackgroundImage: 'assets/img/torah-islamicate.jpg'
+---
+</v>
+      </c>
+      <c r="T14" t="str">
+        <f t="shared" si="7"/>
+        <v># Einführung ins Judentum
+{: .r-fit-text}
+### Wie positionierten sich Rabbiner als die Wahren gegenüber Karäern und Muslimen?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Gründe nennen, warum die Rabbiner nicht als alleinige Repräsentanten des Judentums in den ersten Jahrhunderten u.Z. anzusehen sind.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Einige Unterschiede zwischen Rabbinern, Karäern und Muslimen benennen.</v>
+      </c>
+      <c r="U14" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+Was haben Sie in diesem Kurs gelernt?</v>
+      </c>
+      <c r="V14" t="str">
+        <f t="shared" si="9"/>
+        <v>---
+layout: reveal
+title: 'Wie positionierten sich Rabbiner als die Wahren gegenüber Karäern und Muslimen?'
+author: 'Nathan Gibson'
+session: 10
+tags: [10,slides]
+category: slides
+image: torah-islamicate.jpg
+parallaxBackgroundImage: 'assets/img/torah-islamicate.jpg'
+---
+# Einführung ins Judentum
+{: .r-fit-text}
+### Wie positionierten sich Rabbiner als die Wahren gegenüber Karäern und Muslimen?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Gründe nennen, warum die Rabbiner nicht als alleinige Repräsentanten des Judentums in den ersten Jahrhunderten u.Z. anzusehen sind.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Einige Unterschiede zwischen Rabbinern, Karäern und Muslimen benennen.
+## Lektüre
+## Diskussion
+## Vorschau
+Was haben Sie in diesem Kurs gelernt?</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="3">
         <v>11</v>
       </c>
@@ -1430,7 +2417,7 @@
         <v>70</v>
       </c>
       <c r="L15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v>11-Rückblick</v>
       </c>
       <c r="M15" s="9"/>
@@ -1450,8 +2437,92 @@
 level: overview
 ---</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R15" t="str">
+        <f t="shared" ref="R15" si="11">_xlfn.REGEXREPLACE(D15,"\.md","-slides.md")</f>
+        <v>2025-07-24-11-slides.md</v>
+      </c>
+      <c r="S15" t="str">
+        <f t="shared" ref="S15" si="12">"---
+layout: reveal
+title: '"&amp;G15&amp;"'
+author: 'Nathan Gibson'
+session: "&amp;B15&amp;"
+tags: ["&amp;B15&amp;",slides]
+category: slides
+image: "&amp;K15&amp;"
+parallaxBackgroundImage: 'assets/img/"&amp;K15&amp;"'
+---
+"</f>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Was haben Sie in diesem Kurs gelernt?'
+author: 'Nathan Gibson'
+session: 11
+tags: [11,slides]
+category: slides
+image: scroll.jpg
+parallaxBackgroundImage: 'assets/img/scroll.jpg'
+---
+</v>
+      </c>
+      <c r="T15" t="str">
+        <f t="shared" si="7"/>
+        <v># Einführung ins Judentum
+{: .r-fit-text}
+### Was haben Sie in diesem Kurs gelernt?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Einige Unterschiede zwischen Rabbinern, Karäern und Muslimen benennen.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Das im Kurs neu erworbene Wissen zusammenfassen und festigen.</v>
+      </c>
+      <c r="U15" t="str">
+        <f t="shared" ref="U15" si="13">"
+## Lektüre
+## Diskussion
+## Vorschau
+"&amp;G16</f>
+        <v xml:space="preserve">
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
+      <c r="V15" t="str">
+        <f t="shared" ref="V15" si="14">_xlfn.CONCAT(S15:U15)</f>
+        <v xml:space="preserve">---
+layout: reveal
+title: 'Was haben Sie in diesem Kurs gelernt?'
+author: 'Nathan Gibson'
+session: 11
+tags: [11,slides]
+category: slides
+image: scroll.jpg
+parallaxBackgroundImage: 'assets/img/scroll.jpg'
+---
+# Einführung ins Judentum
+{: .r-fit-text}
+### Was haben Sie in diesem Kurs gelernt?
+Sommersemester 2025
+Prof. Dr. Nathan Gibson
+## 📈 Rückblick: Lernziel
+Einige Unterschiede zwischen Rabbinern, Karäern und Muslimen benennen.
+## 📈 Rückblick: 
+## Projekt
+## Einleitung
+## Heutiges Lernziel
+Das im Kurs neu erworbene Wissen zusammenfassen und festigen.
+## Lektüre
+## Diskussion
+## Vorschau
+</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
       <c r="E16" s="4"/>
     </row>
     <row r="17" spans="5:10" x14ac:dyDescent="0.2">

</xml_diff>